<commit_message>
feat(phase7): regenerate spreadsheet against the improved alignment
Carries phase 5 / phase 6 alignment improvements forward and re-runs
generate_spreadsheet.py. The spreadsheet still contains 346 rows (one
per LLM finding) but more of them are correctly resolved to UDB names:

  Already named in UDB  : 87 rows
  New (unnamed)         : 259 rows
  needs-review hints    : 3 rows (LLM finding legitimately covers
                                  multiple UDB variants)

The "needs review" rows are an honest signal: when a single LLM
extraction maps to a curated one-to-many UDB group (e.g.
REPORT_VA_IN_MTVAL_ON_*), the spreadsheet flags it for human review
rather than silently picking one variant.
</commit_message>
<xml_diff>
--- a/param_extraction/data/parameters.xlsx
+++ b/param_extraction/data/parameters.xlsx
@@ -2551,7 +2551,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>newly discovered</t>
+          <t>needs review: multiple UDB matches (REPORT_GPA_IN_HTVAL_ON_GUEST_PAGE_FAULT, REPORT_GPA_IN_TVAL_ON_INSTRUCTION_GUEST_PAGE_FAULT, REPORT_GPA_IN_TVAL_ON_INTERMEDIATE_GUEST_PAGE_FAULT, REPORT_GPA_IN_TVAL_ON_LOAD_GUEST_PAGE_FAULT, REPORT_GPA_IN_TVAL_ON_STORE_AMO_GUEST_PAGE_FAULT)</t>
         </is>
       </c>
     </row>
@@ -3058,12 +3058,12 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>MSTATUS_VS_LEGAL_VALUES</t>
+          <t>MISELECT_LEGAL_VALUES</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>aligned via fuzzy_name to UDB MSTATUS_VS_LEGAL_VALUES</t>
+          <t>newly discovered</t>
         </is>
       </c>
     </row>
@@ -6683,7 +6683,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>newly discovered</t>
+          <t>needs review: multiple UDB matches (TRAP_ON_ECALL_FROM_M, TRAP_ON_ECALL_FROM_S, TRAP_ON_ECALL_FROM_U, TRAP_ON_ECALL_FROM_VS)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(phase8): propagate alignment lift; tag report and patch unchanged in scope
Carries the curated one-to-many groups, stem matching, regenerated
analysis (v1 + v2) and the refreshed spreadsheet forward to phase 8.
The Phase 8 tagging report itself stays at 328 tags inserted across 48
files with 18 unmatched rows -- tag placement is driven by the
spec-excerpt match, not by the UDB alignment, so this step's output is
unchanged.
</commit_message>
<xml_diff>
--- a/param_extraction/data/parameters.xlsx
+++ b/param_extraction/data/parameters.xlsx
@@ -2551,7 +2551,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>newly discovered</t>
+          <t>needs review: multiple UDB matches (REPORT_GPA_IN_HTVAL_ON_GUEST_PAGE_FAULT, REPORT_GPA_IN_TVAL_ON_INSTRUCTION_GUEST_PAGE_FAULT, REPORT_GPA_IN_TVAL_ON_INTERMEDIATE_GUEST_PAGE_FAULT, REPORT_GPA_IN_TVAL_ON_LOAD_GUEST_PAGE_FAULT, REPORT_GPA_IN_TVAL_ON_STORE_AMO_GUEST_PAGE_FAULT)</t>
         </is>
       </c>
     </row>
@@ -3058,12 +3058,12 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>MSTATUS_VS_LEGAL_VALUES</t>
+          <t>MISELECT_LEGAL_VALUES</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>aligned via fuzzy_name to UDB MSTATUS_VS_LEGAL_VALUES</t>
+          <t>newly discovered</t>
         </is>
       </c>
     </row>
@@ -6683,7 +6683,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>newly discovered</t>
+          <t>needs review: multiple UDB matches (TRAP_ON_ECALL_FROM_M, TRAP_ON_ECALL_FROM_S, TRAP_ON_ECALL_FROM_U, TRAP_ON_ECALL_FROM_VS)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(v3): flag non-verbatim excerpts in the deliverable
Added an excerpt-fidelity check: confirm each excerpt appears (whitespace-
normalized) in its source spec file. Flags 13 rows whose excerpt is a
paraphrase or — for a few params matching the few-shot examples — an echo
of the example text rather than the verbatim chunk. The params are real;
only the quoted wording needs a reviewer's eye. Annotated in notes.

Final deliverable: 201 rows, 12/12 structural audit checks clean, with
over-decomposition and non-verbatim rows explicitly flagged for review.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/param_extraction/data/parameters.xlsx
+++ b/param_extraction/data/parameters.xlsx
@@ -1360,7 +1360,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>newly discovered</t>
+          <t>newly discovered; excerpt not verbatim in spec — verify wording</t>
         </is>
       </c>
     </row>
@@ -1825,7 +1825,11 @@
           <t>KEEP</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>excerpt not verbatim in spec — verify wording</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2037,7 +2041,11 @@
           <t>KEEP</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>excerpt not verbatim in spec — verify wording</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2090,7 +2098,7 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>newly discovered</t>
+          <t>newly discovered; excerpt not verbatim in spec — verify wording</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2259,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>newly discovered</t>
+          <t>newly discovered; excerpt not verbatim in spec — verify wording</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2420,7 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>newly discovered</t>
+          <t>newly discovered; excerpt not verbatim in spec — verify wording</t>
         </is>
       </c>
     </row>
@@ -5449,7 +5457,11 @@
           <t>KEEP</t>
         </is>
       </c>
-      <c r="K94" s="2" t="inlineStr"/>
+      <c r="K94" s="2" t="inlineStr">
+        <is>
+          <t>excerpt not verbatim in spec — verify wording</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -5500,7 +5512,11 @@
           <t>KEEP</t>
         </is>
       </c>
-      <c r="K95" s="2" t="inlineStr"/>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t>excerpt not verbatim in spec — verify wording</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -9095,7 +9111,7 @@
       </c>
       <c r="K162" s="2" t="inlineStr">
         <is>
-          <t>newly discovered</t>
+          <t>newly discovered; excerpt not verbatim in spec — verify wording</t>
         </is>
       </c>
     </row>
@@ -9368,7 +9384,11 @@
           <t>REVIEW_NO_MODAL</t>
         </is>
       </c>
-      <c r="K167" s="2" t="inlineStr"/>
+      <c r="K167" s="2" t="inlineStr">
+        <is>
+          <t>excerpt not verbatim in spec — verify wording</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -9586,7 +9606,7 @@
       </c>
       <c r="K171" s="2" t="inlineStr">
         <is>
-          <t>newly discovered</t>
+          <t>newly discovered; excerpt not verbatim in spec — verify wording</t>
         </is>
       </c>
     </row>
@@ -9641,7 +9661,7 @@
       </c>
       <c r="K172" s="2" t="inlineStr">
         <is>
-          <t>newly discovered</t>
+          <t>newly discovered; excerpt not verbatim in spec — verify wording</t>
         </is>
       </c>
     </row>
@@ -9696,7 +9716,7 @@
       </c>
       <c r="K173" s="2" t="inlineStr">
         <is>
-          <t>newly discovered</t>
+          <t>newly discovered; excerpt not verbatim in spec — verify wording</t>
         </is>
       </c>
     </row>

</xml_diff>